<commit_message>
xA1 ------ m16 dashboard
</commit_message>
<xml_diff>
--- a/utility_core/static/src/Feeder_Migration_Template.xlsx
+++ b/utility_core/static/src/Feeder_Migration_Template.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الفيدرات والخلايا" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="بيانات التهيئة" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تعليمات الاستيراد" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,21 +29,39 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F4E78"/>
-      <sz val="14"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="005D4037"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A237E"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A237E"/>
+      <sz val="14"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -51,8 +70,38 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
+        <fgColor rgb="001A237E"/>
+        <bgColor rgb="001A237E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF8E1"/>
+        <bgColor rgb="00FFF8E1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE0B2"/>
+        <bgColor rgb="00FFE0B2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BBDEFB"/>
+        <bgColor rgb="00BBDEFB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8BBD0"/>
+        <bgColor rgb="00F8BBD0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C8E6C9"/>
+        <bgColor rgb="00C8E6C9"/>
       </patternFill>
     </fill>
   </fills>
@@ -66,33 +115,59 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="00B0BEC5"/>
       </left>
       <right style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="00B0BEC5"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="00B0BEC5"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="00B0BEC5"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -458,272 +533,300 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="72" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="56" customWidth="1" min="4" max="4"/>
-    <col width="31" customWidth="1" min="5" max="5"/>
-    <col width="39" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="144" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
     <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="56" customWidth="1" min="10" max="10"/>
-    <col width="48" customWidth="1" min="11" max="11"/>
-    <col width="32" customWidth="1" min="12" max="12"/>
-    <col width="36" customWidth="1" min="13" max="13"/>
-    <col width="46" customWidth="1" min="14" max="14"/>
-    <col width="29" customWidth="1" min="15" max="15"/>
-    <col width="21" customWidth="1" min="16" max="16"/>
-    <col width="25" customWidth="1" min="17" max="17"/>
+    <col width="55" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="35" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>نموذج استيراد الفيدرات والخلايا - نظام توزيع الكهرباء (Utility ERP)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="25" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>يرجى التاكد من ملء جميع الخانات المعتمدة  |  هل فعال يقبل: نعم / لا  |  رموز المنطقة والفرع تاتي من جدول الترميز  |  القراءة الحالية بالأرقام</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>بيانات المكان والترميز والحالة</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>بيانات الفيدر والخلية</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>بيانات العداد والقراءة</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n"/>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>خيارات الخلية والوصف</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="n"/>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>رمز المنطقة *</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>رمز الفرع *</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>هل فعال؟ *</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>رمز الفيدر / الخلية *</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>اسم الفيدر / الخلية *</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>رقم العداد</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>معامل الضرب للعداد</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>القراءة الحالية</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>خلية إحتساب</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>الوصف</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>HOD</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>MRW</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>H1120-3060</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>خلية الحالي - 3060 - المراوعه -الرئيسية</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>H1120-3060</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="n">
+        <v>12000</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>541.25</v>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>H1120-3060 - خلية الحالي - 3060 - المراوعه -الرئيسية</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>HOD</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>MRW</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>H1101</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>خلية الحالي - 3060 - المراوعه -الخط الشرقي</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>HOD118</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>748.53</v>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="inlineStr">
+        <is>
+          <t>H1101 - خلية الحالي - 3060 - المراوعه -الخط الشرقي</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="I3:J3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="80" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>قالب استيراد وتهيئة الفيدرات والخلايا من النظام السابق - Utility ERP</t>
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>قواعد ملء نموذج الفيدرات والخلايا</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>رمز المنطقة</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>رمز الفرع</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Analytic Account/المعرف</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Analytic Account/اسم العرض</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Analytic Account/رقم العداد</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Analytic Account/معامل الضرب للعداد</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>القراءه السابقة</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>القراءه الحالية</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>تاريخ القراءه</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>وصف</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>Analytic Account/قراءه العداد بدايه الاشتراك</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Analytic Account/خلية إحتساب</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>Analytic Account/الحساب التحليلي</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>Analytic Account/العميل/الاسم</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>الخليه/معامل الضرب للعداد</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>الخليه/رقم العداد</t>
-        </is>
-      </c>
-      <c r="Q2" s="2" t="inlineStr">
-        <is>
-          <t>Analytic Account/مرجع</t>
-        </is>
-      </c>
+      <c r="A2" s="13" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>HOD</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>MRW</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>406888</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>H1120-3060 - خلية الحالي - 3060 - المراوعه -الرئيسية</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>H1120-3060</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>12000</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>531.77</v>
-      </c>
-      <c r="H3" s="3" t="n">
-        <v>541.25</v>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-16 02:05:05</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>H1120-3060 - خلية الحالي - 3060 - المراوعه -الرئيسية</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="n">
-        <v>142.23</v>
-      </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>H1120-3060</t>
-        </is>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>خلية الحالي - 3060 - المراوعه -الرئيسية</t>
-        </is>
-      </c>
-      <c r="O3" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="P3" s="3" t="inlineStr">
-        <is>
-          <t>HOD-102.1</t>
-        </is>
-      </c>
-      <c r="Q3" s="3" t="inlineStr"/>
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>1. الحقول المشار إليها بعلامة (*) إلزامية.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>HOD</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>MRW</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>398548</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>H1101 - خلية الحالي - 3060 - المراوعه -الخط الشرقي</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>HOD118</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>263.12</v>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>748.53</v>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-16 02:05:05</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>H1101 - خلية الحالي - 3060 - المراوعه -الخط الشرقي</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="n">
-        <v>1.72</v>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>H1101</t>
-        </is>
-      </c>
-      <c r="N4" s="3" t="inlineStr">
-        <is>
-          <t>خلية الحالي - 3060 - المراوعه -الخط الشرقي</t>
-        </is>
-      </c>
-      <c r="O4" s="3" t="n">
-        <v>12000</v>
-      </c>
-      <c r="P4" s="3" t="inlineStr">
-        <is>
-          <t>H1120-3060</t>
-        </is>
-      </c>
-      <c r="Q4" s="3" t="inlineStr"/>
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>2. حقل هل فعال يقبل القيمتين: نعم أو لا.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>3. رمزا المنطقة والفرع يجب أن يطابقا جدول الترميز الموجود في النظام.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>4. حقل خلية إحتساب يقبل القيمتين: TRUE أو FALSE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>5. أرقام العدادات وقيم القراءات الحالية والمعاملات تُدخل بالأرقام فقط.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:Q1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
dev ++ ----------- enhance lifecycle replacement respects 13 +1
</commit_message>
<xml_diff>
--- a/utility_core/static/src/Feeder_Migration_Template.xlsx
+++ b/utility_core/static/src/Feeder_Migration_Template.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تعليمات الاستيراد" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'بيانات التهيئة'!$A$4:$L$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'بيانات التهيئة'!$A$4:$M$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -208,7 +208,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -263,6 +263,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -628,7 +634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1004"/>
+  <dimension ref="A1:M1004"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -643,6 +649,7 @@
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="25" customWidth="1" min="11" max="11"/>
     <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
@@ -688,64 +695,69 @@
       <c r="J3" s="15" t="n"/>
     </row>
     <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>رمز المنطقة</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>رمز الفرع</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr">
+      <c r="C4" s="24" t="inlineStr">
         <is>
           <t>هل فعال؟ *</t>
         </is>
       </c>
-      <c r="D4" s="17" t="inlineStr">
+      <c r="D4" s="24" t="inlineStr">
         <is>
           <t>رمز الفيدر / الخلية *</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr">
+      <c r="E4" s="24" t="inlineStr">
         <is>
           <t>اسم الفيدر / الخلية *</t>
         </is>
       </c>
-      <c r="F4" s="17" t="inlineStr">
+      <c r="F4" s="24" t="inlineStr">
         <is>
           <t>رقم العداد</t>
         </is>
       </c>
-      <c r="G4" s="16" t="inlineStr">
+      <c r="G4" s="24" t="inlineStr">
         <is>
           <t>معامل الضرب للعداد</t>
         </is>
       </c>
-      <c r="H4" s="16" t="inlineStr">
+      <c r="H4" s="24" t="inlineStr">
         <is>
           <t>القراءة الحالية</t>
         </is>
       </c>
-      <c r="I4" s="16" t="inlineStr">
+      <c r="I4" s="24" t="inlineStr">
         <is>
           <t>خلية إحتساب</t>
         </is>
       </c>
-      <c r="J4" s="16" t="inlineStr">
+      <c r="J4" s="24" t="inlineStr">
         <is>
           <t>الوصف</t>
         </is>
       </c>
-      <c r="K4" s="18" t="inlineStr">
+      <c r="K4" s="25" t="inlineStr">
         <is>
           <t>معرف الحساب التحليلي</t>
         </is>
       </c>
-      <c r="L4" s="18" t="inlineStr">
+      <c r="L4" s="25" t="inlineStr">
         <is>
           <t>قراءة بداية الاشتراك</t>
+        </is>
+      </c>
+      <c r="M4" s="25" t="inlineStr">
+        <is>
+          <t>منطقة إنتاج؟</t>
         </is>
       </c>
     </row>
@@ -10750,7 +10762,7 @@
       <c r="L1004" s="20" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L4"/>
+  <autoFilter ref="A4:M4"/>
   <mergeCells count="6">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A3:C3"/>
@@ -10759,11 +10771,14 @@
     <mergeCell ref="D3:E3"/>
     <mergeCell ref="I3:J3"/>
   </mergeCells>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="C5:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"نعم,لا,TRUE,FALSE"</formula1>
     </dataValidation>
     <dataValidation sqref="I5:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"نعم,لا,TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="M5:M1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"نعم,لا,TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10777,20 +10792,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="110" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="21" t="inlineStr">
         <is>
-          <t>تعليمات الاستيراد — عقد ترحيل رسمي</t>
+          <t>تعليمات استيراد الفيدرات — عقد v3</t>
         </is>
       </c>
-      <c r="B1" s="22" t="n"/>
+      <c r="B1" s="22" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" s="23" t="inlineStr">
@@ -10800,7 +10815,7 @@
       </c>
       <c r="B2" s="22" t="inlineStr">
         <is>
-          <t>Feeder_Migration_Template</t>
+          <t>feeder</t>
         </is>
       </c>
     </row>
@@ -10811,126 +10826,66 @@
         </is>
       </c>
       <c r="B3" s="22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="23" t="inlineStr">
         <is>
-          <t>نوع الملف</t>
+          <t>الهوية</t>
         </is>
       </c>
       <c r="B4" s="22" t="inlineStr">
         <is>
-          <t>.xlsx فقط — لا تستخدم .xls</t>
+          <t>feeder_code ثم legacy_analytic_id؛ لا تستخدم الاسم أو الوصف.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="23" t="inlineStr">
         <is>
-          <t>الحقول الإلزامية</t>
+          <t>منطقة إنتاج</t>
         </is>
       </c>
       <c r="B5" s="22" t="inlineStr">
         <is>
-          <t>رمز الفيدر / الخلية *، اسم الفيدر / الخلية *، رقم العداد</t>
+          <t>منطقة إنتاج؟ = نعم يحوّل feeder_type إلى production_area. لا يتم الاستدلال من الاسم أو الوصف.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="23" t="inlineStr">
         <is>
-          <t>الحقول الاختيارية</t>
+          <t>القراءات</t>
         </is>
       </c>
       <c r="B6" s="22" t="inlineStr">
         <is>
-          <t>تُترك فارغة عند عدم توفرها، ولا تحذف العناوين</t>
+          <t>current_reading له الأولوية على opening_reading؛ الفراغ لا ينشئ قراءة.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="23" t="inlineStr">
         <is>
-          <t>قواعد الهوية</t>
+          <t>القيم</t>
         </is>
       </c>
       <c r="B7" s="22" t="inlineStr">
         <is>
-          <t>feeder_code ثم legacy_analytic_id؛ لا تستخدم الاسم أو الوصف.</t>
+          <t>المعامل أكبر من صفر، والقراءات غير سالبة. الفراغ ليس صفراً.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="23" t="inlineStr">
         <is>
-          <t>القراءات</t>
+          <t>تنبيه</t>
         </is>
       </c>
       <c r="B8" s="22" t="inlineStr">
         <is>
-          <t>current_reading له الأولوية على opening_reading؛ الفراغ لا ينشئ قراءة.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="23" t="inlineStr">
-        <is>
-          <t>القيم المنطقية</t>
-        </is>
-      </c>
-      <c r="B9" s="22" t="inlineStr">
-        <is>
-          <t>TRUE/FALSE أو نعم/لا أو 1/0 أو yes/no فقط؛ القيمة غير المعروفة خطأ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="23" t="inlineStr">
-        <is>
-          <t>الطور</t>
-        </is>
-      </c>
-      <c r="B10" s="22" t="inlineStr">
-        <is>
-          <t>single أو three فقط؛ القيمة غير المعروفة خطأ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="23" t="inlineStr">
-        <is>
-          <t>الأرقام</t>
-        </is>
-      </c>
-      <c r="B11" s="22" t="inlineStr">
-        <is>
-          <t>القراءات والمعاملات أرقام حقيقية غير سالبة؛ الفراغ ليس صفرًا، والصفر قيمة صحيحة.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="23" t="inlineStr">
-        <is>
-          <t>تنبيه</t>
-        </is>
-      </c>
-      <c r="B12" s="22" t="inlineStr">
-        <is>
-          <t>لا تغيّر أسماء العناوين، لا تدمج خلايا البيانات، لا تضف صيغًا، وحافظ على الأصفار البادئة للمعرفات.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="23" t="inlineStr">
-        <is>
-          <t>Example</t>
-        </is>
-      </c>
-      <c r="B13" s="22" t="inlineStr">
-        <is>
-          <t>feeder_code=FDR-001، current_reading=0.</t>
+          <t>لا تغيّر العناوين، لا تدمج خلايا Data، لا تستخدم صيغاً، واحفظ الأصفار البادئة.</t>
         </is>
       </c>
     </row>

</xml_diff>